<commit_message>
updated node metrics & pipeline distances (hypothetical transport hub added)
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_railway.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_railway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ykk/Documents/GitHub/AdOpT-NET0_XiaoY/southern_europe/italy_data/network_capex_metrics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF102B20-A4F4-A94F-8C99-4D7C25CF2EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A88851-F5D0-4A4A-825F-0DD3C6B25359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="6640" windowWidth="30240" windowHeight="10280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1580" windowWidth="30240" windowHeight="15340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="gamma1" sheetId="1" r:id="rId1"/>
@@ -6298,10 +6298,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AS45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.2">
       <c r="B1">
         <v>1</v>
       </c>
@@ -6431,8 +6431,11 @@
       <c r="AR1">
         <v>43</v>
       </c>
+      <c r="AS1">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6566,8 +6569,11 @@
       <c r="AR2">
         <v>0</v>
       </c>
+      <c r="AS2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6700,8 +6706,11 @@
       <c r="AR3">
         <v>0</v>
       </c>
+      <c r="AS3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -6835,8 +6844,11 @@
       <c r="AR4">
         <v>0</v>
       </c>
+      <c r="AS4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6969,8 +6981,11 @@
       <c r="AR5">
         <v>0</v>
       </c>
+      <c r="AS5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7103,8 +7118,11 @@
       <c r="AR6">
         <v>0</v>
       </c>
+      <c r="AS6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -7237,8 +7255,11 @@
       <c r="AR7">
         <v>0</v>
       </c>
+      <c r="AS7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7373,8 +7394,11 @@
       <c r="AR8">
         <v>0</v>
       </c>
+      <c r="AS8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7506,8 +7530,11 @@
       <c r="AR9">
         <v>0</v>
       </c>
+      <c r="AS9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -7640,8 +7667,11 @@
       <c r="AR10">
         <v>0</v>
       </c>
+      <c r="AS10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -7774,8 +7804,11 @@
       <c r="AR11">
         <v>0</v>
       </c>
+      <c r="AS11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -7909,8 +7942,11 @@
       <c r="AR12">
         <v>0</v>
       </c>
+      <c r="AS12">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -8043,8 +8079,11 @@
       <c r="AR13">
         <v>0</v>
       </c>
+      <c r="AS13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -8177,8 +8216,11 @@
       <c r="AR14">
         <v>0</v>
       </c>
+      <c r="AS14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -8311,8 +8353,11 @@
       <c r="AR15">
         <v>0</v>
       </c>
+      <c r="AS15">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -8446,8 +8491,11 @@
       <c r="AR16">
         <v>0</v>
       </c>
+      <c r="AS16">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -8580,8 +8628,11 @@
       <c r="AR17">
         <v>0</v>
       </c>
+      <c r="AS17">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -8714,8 +8765,11 @@
       <c r="AR18">
         <v>0</v>
       </c>
+      <c r="AS18">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -8848,8 +8902,11 @@
       <c r="AR19">
         <v>0</v>
       </c>
+      <c r="AS19">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -8982,8 +9039,11 @@
       <c r="AR20">
         <v>0</v>
       </c>
+      <c r="AS20">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -9116,8 +9176,11 @@
       <c r="AR21">
         <v>0</v>
       </c>
+      <c r="AS21">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -9250,8 +9313,11 @@
       <c r="AR22">
         <v>0</v>
       </c>
+      <c r="AS22">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -9384,8 +9450,11 @@
       <c r="AR23">
         <v>0</v>
       </c>
+      <c r="AS23">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -9519,8 +9588,11 @@
       <c r="AR24">
         <v>0</v>
       </c>
+      <c r="AS24">
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -9653,8 +9725,11 @@
       <c r="AR25">
         <v>0</v>
       </c>
+      <c r="AS25">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -9787,8 +9862,11 @@
       <c r="AR26">
         <v>0</v>
       </c>
+      <c r="AS26">
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -9922,8 +10000,11 @@
       <c r="AR27">
         <v>0</v>
       </c>
+      <c r="AS27">
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -10056,8 +10137,11 @@
       <c r="AR28">
         <v>0</v>
       </c>
+      <c r="AS28">
+        <v>0</v>
+      </c>
     </row>
-    <row r="29" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -10190,8 +10274,11 @@
       <c r="AR29">
         <v>0</v>
       </c>
+      <c r="AS29">
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -10324,8 +10411,11 @@
       <c r="AR30">
         <v>0</v>
       </c>
+      <c r="AS30">
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -10459,8 +10549,11 @@
       <c r="AR31">
         <v>0</v>
       </c>
+      <c r="AS31">
+        <v>0</v>
+      </c>
     </row>
-    <row r="32" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -10593,8 +10686,11 @@
       <c r="AR32">
         <v>0</v>
       </c>
+      <c r="AS32">
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -10727,8 +10823,11 @@
       <c r="AR33">
         <v>0</v>
       </c>
+      <c r="AS33">
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -10861,8 +10960,11 @@
       <c r="AR34">
         <v>0</v>
       </c>
+      <c r="AS34">
+        <v>0</v>
+      </c>
     </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -10997,8 +11099,11 @@
       <c r="AR35">
         <v>0</v>
       </c>
+      <c r="AS35">
+        <v>0</v>
+      </c>
     </row>
-    <row r="36" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -11131,8 +11236,11 @@
       <c r="AR36">
         <v>0</v>
       </c>
+      <c r="AS36">
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -11265,8 +11373,11 @@
       <c r="AR37">
         <v>0</v>
       </c>
+      <c r="AS37">
+        <v>0</v>
+      </c>
     </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -11399,8 +11510,11 @@
       <c r="AR38">
         <v>0</v>
       </c>
+      <c r="AS38">
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -11534,8 +11648,11 @@
       <c r="AR39">
         <v>0</v>
       </c>
+      <c r="AS39">
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -11668,8 +11785,11 @@
       <c r="AR40">
         <v>0</v>
       </c>
+      <c r="AS40">
+        <v>0</v>
+      </c>
     </row>
-    <row r="41" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -11802,8 +11922,11 @@
       <c r="AR41">
         <v>0</v>
       </c>
+      <c r="AS41">
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -11937,8 +12060,11 @@
       <c r="AR42">
         <v>0</v>
       </c>
+      <c r="AS42">
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -12071,8 +12197,11 @@
       <c r="AR43">
         <v>0</v>
       </c>
+      <c r="AS43">
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -12205,9 +12334,149 @@
       <c r="AR44">
         <v>0</v>
       </c>
+      <c r="AS44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
+      <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
+        <v>0</v>
+      </c>
+      <c r="N45">
+        <v>0</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
+        <v>0</v>
+      </c>
+      <c r="Q45">
+        <v>0</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+      <c r="S45">
+        <v>0</v>
+      </c>
+      <c r="T45">
+        <v>0</v>
+      </c>
+      <c r="U45">
+        <v>0</v>
+      </c>
+      <c r="V45">
+        <v>0</v>
+      </c>
+      <c r="W45">
+        <v>0</v>
+      </c>
+      <c r="X45">
+        <v>0</v>
+      </c>
+      <c r="Y45">
+        <v>0</v>
+      </c>
+      <c r="Z45">
+        <v>0</v>
+      </c>
+      <c r="AA45">
+        <v>0</v>
+      </c>
+      <c r="AB45">
+        <v>0</v>
+      </c>
+      <c r="AC45">
+        <v>0</v>
+      </c>
+      <c r="AD45">
+        <v>0</v>
+      </c>
+      <c r="AE45">
+        <v>0</v>
+      </c>
+      <c r="AF45">
+        <v>0</v>
+      </c>
+      <c r="AG45">
+        <v>0</v>
+      </c>
+      <c r="AH45">
+        <v>0</v>
+      </c>
+      <c r="AI45">
+        <v>0</v>
+      </c>
+      <c r="AJ45">
+        <v>0</v>
+      </c>
+      <c r="AK45">
+        <v>0</v>
+      </c>
+      <c r="AL45">
+        <v>0</v>
+      </c>
+      <c r="AM45">
+        <v>0</v>
+      </c>
+      <c r="AN45">
+        <v>0</v>
+      </c>
+      <c r="AO45">
+        <v>0</v>
+      </c>
+      <c r="AP45">
+        <v>0</v>
+      </c>
+      <c r="AQ45">
+        <v>0</v>
+      </c>
+      <c r="AR45">
+        <v>0</v>
+      </c>
+      <c r="AS45">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:AR44">
+  <conditionalFormatting sqref="B2:AS45">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>